<commit_message>
csp solver done and testrun successful
</commit_message>
<xml_diff>
--- a/backend/excel_reader/testcase_1.xlsx
+++ b/backend/excel_reader/testcase_1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ashwin\timetable-ai\backend\app\excel_reader\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ashwin\Timetable AI\timetable-ai\backend\excel_reader\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D173EC4-2109-4C63-8516-9DAD6D09DF4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{139D90F8-8B86-4333-A8C8-A761EFD51D20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{99D41510-FAAC-44E4-A3FB-31B80A49CAE5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{99D41510-FAAC-44E4-A3FB-31B80A49CAE5}"/>
   </bookViews>
   <sheets>
     <sheet name="Staff" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="87">
   <si>
     <t>staff_name</t>
   </si>
@@ -238,9 +238,6 @@
   </si>
   <si>
     <t>Aptitude</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PL309 </t>
   </si>
   <si>
     <t>Programming Lab</t>
@@ -980,7 +977,7 @@
         <v>38</v>
       </c>
       <c r="B10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C10" t="s">
         <v>25</v>
@@ -994,7 +991,7 @@
         <v>37</v>
       </c>
       <c r="B11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C11" t="s">
         <v>25</v>
@@ -1243,16 +1240,16 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" t="s">
         <v>69</v>
       </c>
-      <c r="B10" t="s">
-        <v>70</v>
-      </c>
       <c r="C10" t="s">
         <v>25</v>
       </c>
       <c r="D10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" t="s">
         <v>27</v>
@@ -1260,16 +1257,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" t="s">
         <v>71</v>
       </c>
-      <c r="B11" t="s">
-        <v>72</v>
-      </c>
       <c r="C11" t="s">
         <v>25</v>
       </c>
       <c r="D11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" t="s">
         <v>27</v>
@@ -1318,7 +1315,7 @@
         <v>50</v>
       </c>
       <c r="B2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C2">
         <v>70</v>
@@ -1338,7 +1335,7 @@
         <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C3">
         <v>70</v>
@@ -1355,10 +1352,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C4">
         <v>35</v>
@@ -1375,10 +1372,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C5">
         <v>40</v>
@@ -1392,10 +1389,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C6">
         <v>60</v>
@@ -1584,7 +1581,7 @@
         <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C2">
         <v>8</v>
@@ -1598,7 +1595,7 @@
         <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -1612,7 +1609,7 @@
         <v>31</v>
       </c>
       <c r="B4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4">
         <v>8</v>
@@ -1626,7 +1623,7 @@
         <v>32</v>
       </c>
       <c r="B5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -1640,10 +1637,10 @@
         <v>33</v>
       </c>
       <c r="B6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D6">
         <v>2</v>
@@ -1654,7 +1651,7 @@
         <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -1668,7 +1665,7 @@
         <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -1682,7 +1679,7 @@
         <v>36</v>
       </c>
       <c r="B9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -1696,7 +1693,7 @@
         <v>38</v>
       </c>
       <c r="B10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -1710,7 +1707,7 @@
         <v>37</v>
       </c>
       <c r="B11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C11">
         <v>8</v>

</xml_diff>